<commit_message>
bug: log BUG_030,031,032 for JD Match Module
</commit_message>
<xml_diff>
--- a/Documentation/BugReports/BugReport.xlsx
+++ b/Documentation/BugReports/BugReport.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="237">
   <si>
     <t>BUG_ID</t>
   </si>
@@ -755,12 +755,74 @@
   <si>
     <t>Retested after fix. Issue verified successfully. Resume deletion endpoint now requires the correct HTTP method and validates CSRF protection before processing the request. Cross-origin forged requests are rejected, and unauthorized resume deletion is no longer possible.</t>
   </si>
+  <si>
+    <t>BUG_030</t>
+  </si>
+  <si>
+    <t>JD Match analysis produces inconsistent/non-reproducible results for identical resume + JD input</t>
+  </si>
+  <si>
+    <t>1. Upload resume (MIS_Executive_ATS_Resume.pdf).
+2. Paste a fixed Job Description (MIS Executive - Fresher role, listing MS Excel, MS Word, MS Outlook, data entry, VLOOKUP, Pivot Table as required skills).
+3. Click Analyze Match.
+4. Repeat steps 1-3 two more times with the exact same resume and exact same JD text, without changing any input.</t>
+  </si>
+  <si>
+    <t>Given identical resume and JD input, the match percentage, matched_skills, and missing_skills should be the same (or nearly identical) across repeated runs, since the underlying facts (what's in the resume vs what's in the JD) have not changed.</t>
+  </si>
+  <si>
+    <t>Three consecutive runs with identical input produced three very different results:
+Run 1: 0.0% match, 0 matched, 0 missing — AI Analysis Feedback showed a raw error instead of a real result (see BUG_031).
+Run 2: 71.4% match, 5 matched (MS Excel, MS Word, Data Entry, Attention to Detail, Communication), 2 missing (VLOOKUP, Pivot Table).
+Run 3: 40.0% match, 2 matched (MS Excel, MS Word), 3 missing (VLOOKUP, Pivot Table, data entry skills).</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>BUG_031</t>
+  </si>
+  <si>
+    <t>AI Analysis Feedback displays a raw JSON parsing error message instead of a graceful fallback</t>
+  </si>
+  <si>
+    <t>1. Upload resume.
+2. Paste JD and click Analyze Match.
+3. If the Groq API response is malformed/truncated, observe the AI Analysis Feedback section.</t>
+  </si>
+  <si>
+    <t>If AI analysis fails for any reason (malformed LLM response, API error, etc.), the UI should show a clean, user-friendly message (e.g. "We couldn't fully analyze this JD, please try again") and the match score/skills sections should not silently report 0%/empty as if that were a genuine result.</t>
+  </si>
+  <si>
+    <t>The AI Analysis Feedback section displayed the raw Python exception text verbatim: "Analysis failed: Expecting ',' delimiter: line 1 column 724 (char 723)". The JD Match Result card simultaneously showed 0.0% match with 0 matched/0 missing skills, indistinguishable from a genuine "no skills found" case — the user has no way to tell this was a system error versus an actual analysis result.</t>
+  </si>
+  <si>
+    <t>BUG_032</t>
+  </si>
+  <si>
+    <t>JD Match silently drops an explicitly-stated JD skill from both matched_skills and missing_skills</t>
+  </si>
+  <si>
+    <t>1. Upload resume (MIS_Executive_ATS_Resume.pdf).
+2. Paste JD for MIS Executive (Fresher) role, which explicitly lists "Basic knowledge of MS Word and Outlook" as a required skill, alongside MS Excel, VLOOKUP, Pivot Table, and Data Entry.
+3. Click Analyze Match.
+4. Count total skills covered across matched_skills + missing_skills and compare against the number of distinct skills explicitly named in the JD.</t>
+  </si>
+  <si>
+    <t>Every skill explicitly named in the JD should be classified into exactly one of matched_skills or missing_skills, so the two lists together account for all JD requirements (6 skills in this JD).</t>
+  </si>
+  <si>
+    <t>Result showed 3 matched (MS Excel, MS Word, Data Entry) + 2 missing (VLOOKUP, Pivot Table) = 5 of 6 JD skills. "MS Outlook" was not present in either list, even though the AI Analysis Feedback text itself referenced it ("...lacks specific examples of experience with MS Outlook"), confirming the model recognized it as a JD requirement but never placed it in matched_skills or missing_skills.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -780,6 +842,11 @@
     </font>
     <font>
       <sz val="10.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
@@ -824,7 +891,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -856,6 +923,12 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -2583,17 +2656,37 @@
       <c r="Z30" s="10"/>
     </row>
     <row r="31">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
+      <c r="A31" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="K31" s="9" t="s">
+        <v>226</v>
+      </c>
       <c r="L31" s="10"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
@@ -2611,17 +2704,37 @@
       <c r="Z31" s="10"/>
     </row>
     <row r="32">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10"/>
+      <c r="A32" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="K32" s="9" t="s">
+        <v>226</v>
+      </c>
       <c r="L32" s="10"/>
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
@@ -2639,17 +2752,37 @@
       <c r="Z32" s="10"/>
     </row>
     <row r="33">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
+      <c r="A33" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="J33" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>226</v>
+      </c>
       <c r="L33" s="10"/>
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
@@ -29748,7 +29881,7 @@
     <dataValidation type="list" allowBlank="1" sqref="K2:K30">
       <formula1>"Open,Close"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B30">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B33">
       <formula1>"Bug,Enhancement"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H2:I24">

</xml_diff>